<commit_message>
Add credit price (priceCheck) support across product model, forms, cart, and import
Products now carry a separate cash and check/credit price. Adds the field
to the schema, admin create/edit forms, bulk import (with template columns),
and wires payment-type-aware price display through product cards, product
detail, cart, and order building. Also fixes the bulk importer overwriting
whole product documents (wiping fields like promotion) and zeroing priceCheck
on blank cells, and makes MongoDB connection retry instead of exiting on
initial failure.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/templates/price-update-template.xlsx
+++ b/server/templates/price-update-template.xlsx
@@ -12,12 +12,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>کد محصول</t>
   </si>
   <si>
     <t>قیمت (تومان)</t>
+  </si>
+  <si>
+    <t>قیمت اعتباری (تومان)</t>
   </si>
   <si>
     <t>موجودی</t>
@@ -451,37 +454,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="18" customWidth="1"/>
+    <col min="1" max="2" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
         <v>5</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -495,36 +502,36 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>